<commit_message>
W3 D5- Conditional Formatting and visualas Analysis
</commit_message>
<xml_diff>
--- a/Month-01-Excel/Week-03/Day-04/W3-D4-Business-Analysis-PivotTables.xlsx
+++ b/Month-01-Excel/Week-03/Day-04/W3-D4-Business-Analysis-PivotTables.xlsx
@@ -8,18 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\4_MONTH\4-Month-Data-Analyst-Journey\Month-01-Excel\Week-03\Day-04\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D88BAEA4-A75B-4CE5-8741-C9E180D92CFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAB7959A-A806-41FF-8463-61675D76FD27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw data" sheetId="2" r:id="rId1"/>
     <sheet name="Business_Analysis" sheetId="1" r:id="rId2"/>
-    <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
+    <sheet name="Notes" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="22" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -455,12 +455,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -475,13 +474,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -492,24 +484,24 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="3">
     <dxf>
       <alignment horizontal="left"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
     </dxf>
     <dxf>
       <alignment horizontal="left"/>
@@ -764,7 +756,554 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D50F9526-A2B9-4D1F-B758-89BA7EA6CD08}" name="PivotTable11" cacheId="22" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{08D20DB3-2DB0-4E48-BAA4-00B62E849827}" name="PivotTable9" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A58:B64" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="8">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="2"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item x="0"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Order_ID" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable10.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{49882A7B-EB71-445A-9CBF-CFFFD2FE402D}" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A25:B29" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="8">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Quantity" fld="6" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1476AB5D-4A61-4977-9D3F-82DD3E2871ED}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A16:B22" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="8">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="2"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item x="0"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Sales" fld="7" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4F5687CC-4202-44B1-8A58-848D42383AD2}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A9:B13" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="8">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="4"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Sales" fld="7" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{CEC1C61A-CD7A-4A55-AD5C-1F238C1D2447}" name="PivotTable8" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A50:C55" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="8">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="5">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" showAll="0">
+      <items count="12">
+        <item x="4"/>
+        <item x="1"/>
+        <item x="10"/>
+        <item x="7"/>
+        <item x="2"/>
+        <item x="9"/>
+        <item x="6"/>
+        <item x="3"/>
+        <item x="8"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="5"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="2">
+    <dataField name="Sum of Quantity" fld="6" baseField="0" baseItem="0"/>
+    <dataField name="Sum of Sales" fld="7" baseField="5" baseItem="0"/>
+  </dataFields>
+  <conditionalFormats count="1">
+    <conditionalFormat priority="2">
+      <pivotAreas count="1">
+        <pivotArea type="data" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="1"/>
+            </reference>
+            <reference field="5" count="4">
+              <x v="0"/>
+              <x v="1"/>
+              <x v="2"/>
+              <x v="3"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </pivotAreas>
+    </conditionalFormat>
+  </conditionalFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{19AD61D7-E742-4494-8F03-50C26C9DF995}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A2:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="8">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Sales" fld="7" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D3E8DC91-D9DE-4282-9822-1D82C45BD30F}" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A40:E47" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="8">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="2"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item x="0"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="4">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="4"/>
+  </colFields>
+  <colItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Sales" fld="7" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EC896C35-2235-45DC-8917-1BA2FB7006BD}" name="PivotTable6" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A32:C37" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="8">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="4">
+        <item h="1" x="1"/>
+        <item x="0"/>
+        <item h="1" x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="4"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Sales" fld="7" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D50F9526-A2B9-4D1F-B758-89BA7EA6CD08}" name="PivotTable11" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A76:E83" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="8">
     <pivotField showAll="0"/>
@@ -836,14 +1375,14 @@
     <dataField name="Sum of Sales" fld="7" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="3">
-    <format dxfId="3">
+    <format dxfId="2">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="2">
+    <format dxfId="1">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
@@ -886,63 +1425,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable10.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{19AD61D7-E742-4494-8F03-50C26C9DF995}" name="PivotTable1" cacheId="22" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A2:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="8">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="4">
-        <item x="1"/>
-        <item x="0"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="3"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of Sales" fld="7" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8E0D50BB-2FA9-472D-80A3-F7FE22F0E5A9}" name="PivotTable10" cacheId="22" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8E0D50BB-2FA9-472D-80A3-F7FE22F0E5A9}" name="PivotTable10" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A67:I73" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="8">
     <pivotField showAll="0"/>
@@ -1058,498 +1542,6 @@
     <dataField name="Sum of Sales" fld="7" baseField="0" baseItem="0"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight14" showRowHeaders="1" showColHeaders="1" showRowStripes="1" showColStripes="1" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{08D20DB3-2DB0-4E48-BAA4-00B62E849827}" name="PivotTable9" cacheId="22" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A58:B64" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="8">
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="2"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item x="0"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="2"/>
-  </rowFields>
-  <rowItems count="6">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Count of Order_ID" fld="0" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{CEC1C61A-CD7A-4A55-AD5C-1F238C1D2447}" name="PivotTable8" cacheId="22" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A50:C55" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="8">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="5">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0">
-      <items count="12">
-        <item x="4"/>
-        <item x="1"/>
-        <item x="10"/>
-        <item x="7"/>
-        <item x="2"/>
-        <item x="9"/>
-        <item x="6"/>
-        <item x="3"/>
-        <item x="8"/>
-        <item x="5"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="5"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="-2"/>
-  </colFields>
-  <colItems count="2">
-    <i>
-      <x/>
-    </i>
-    <i i="1">
-      <x v="1"/>
-    </i>
-  </colItems>
-  <dataFields count="2">
-    <dataField name="Sum of Quantity" fld="6" baseField="0" baseItem="0"/>
-    <dataField name="Sum of Sales" fld="7" baseField="5" baseItem="0"/>
-  </dataFields>
-  <conditionalFormats count="1">
-    <conditionalFormat priority="2">
-      <pivotAreas count="1">
-        <pivotArea type="data" collapsedLevelsAreSubtotals="1" fieldPosition="0">
-          <references count="2">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="1"/>
-            </reference>
-            <reference field="5" count="4">
-              <x v="0"/>
-              <x v="1"/>
-              <x v="2"/>
-              <x v="3"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </pivotAreas>
-    </conditionalFormat>
-  </conditionalFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D3E8DC91-D9DE-4282-9822-1D82C45BD30F}" name="PivotTable7" cacheId="22" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A40:E47" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="8">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="2"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item x="0"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisCol" showAll="0">
-      <items count="4">
-        <item x="1"/>
-        <item x="0"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="2"/>
-  </rowFields>
-  <rowItems count="6">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="4"/>
-  </colFields>
-  <colItems count="4">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of Sales" fld="7" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EC896C35-2235-45DC-8917-1BA2FB7006BD}" name="PivotTable6" cacheId="22" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A32:C37" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="8">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="4">
-        <item x="1"/>
-        <item x="0"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisCol" showAll="0">
-      <items count="4">
-        <item h="1" x="1"/>
-        <item x="0"/>
-        <item h="1" x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="3"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="4"/>
-  </colFields>
-  <colItems count="2">
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of Sales" fld="7" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{49882A7B-EB71-445A-9CBF-CFFFD2FE402D}" name="PivotTable5" cacheId="22" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A25:B29" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="8">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="4">
-        <item x="1"/>
-        <item x="0"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="3"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of Quantity" fld="6" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1476AB5D-4A61-4977-9D3F-82DD3E2871ED}" name="PivotTable3" cacheId="22" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A16:B22" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="8">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="2"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item x="0"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="2"/>
-  </rowFields>
-  <rowItems count="6">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of Sales" fld="7" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4F5687CC-4202-44B1-8A58-848D42383AD2}" name="PivotTable2" cacheId="22" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A9:B13" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="8">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="4">
-        <item x="1"/>
-        <item x="0"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="4"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of Sales" fld="7" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
       <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
@@ -1859,392 +1851,392 @@
       </c>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="3">
         <v>46031</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="2">
         <v>2</v>
       </c>
-      <c r="H2" s="3">
+      <c r="H2" s="2">
         <v>110000</v>
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="3">
         <v>46062</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="2">
         <v>5</v>
       </c>
-      <c r="H3" s="3">
+      <c r="H3" s="2">
         <v>6000</v>
       </c>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="3">
         <v>46090</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="2">
         <v>3</v>
       </c>
-      <c r="H4" s="3">
+      <c r="H4" s="2">
         <v>15000</v>
       </c>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5" s="3">
         <v>46121</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="G5" s="3">
+      <c r="G5" s="2">
         <v>2</v>
       </c>
-      <c r="H5" s="3">
+      <c r="H5" s="2">
         <v>36000</v>
       </c>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="3">
         <v>46151</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G6" s="3">
+      <c r="G6" s="2">
         <v>4</v>
       </c>
-      <c r="H6" s="3">
+      <c r="H6" s="2">
         <v>4800</v>
       </c>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="3">
         <v>46182</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="3">
+      <c r="G7" s="2">
         <v>1</v>
       </c>
-      <c r="H7" s="3">
+      <c r="H7" s="2">
         <v>55000</v>
       </c>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B8" s="3">
         <v>46212</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="F8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G8" s="3">
+      <c r="G8" s="2">
         <v>5</v>
       </c>
-      <c r="H8" s="3">
+      <c r="H8" s="2">
         <v>25000</v>
       </c>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B9" s="3">
         <v>46243</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G9" s="3">
+      <c r="G9" s="2">
         <v>8</v>
       </c>
-      <c r="H9" s="3">
+      <c r="H9" s="2">
         <v>9600</v>
       </c>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="4">
+      <c r="B10" s="3">
         <v>46274</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="F10" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="G10" s="3">
+      <c r="G10" s="2">
         <v>3</v>
       </c>
-      <c r="H10" s="3">
+      <c r="H10" s="2">
         <v>54000</v>
       </c>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="4">
+      <c r="B11" s="3">
         <v>46304</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G11" s="3">
+      <c r="G11" s="2">
         <v>4</v>
       </c>
-      <c r="H11" s="3">
+      <c r="H11" s="2">
         <v>20000</v>
       </c>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B12" s="4">
+      <c r="B12" s="3">
         <v>46335</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F12" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G12" s="3">
+      <c r="G12" s="2">
         <v>2</v>
       </c>
-      <c r="H12" s="3">
+      <c r="H12" s="2">
         <v>110000</v>
       </c>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="4">
+      <c r="B13" s="3">
         <v>46365</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="E13" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="F13" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G13" s="3">
+      <c r="G13" s="2">
         <v>6</v>
       </c>
-      <c r="H13" s="3">
+      <c r="H13" s="2">
         <v>7200</v>
       </c>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E14" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="F14" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="G14" s="3">
+      <c r="G14" s="2">
         <v>2</v>
       </c>
-      <c r="H14" s="3">
+      <c r="H14" s="2">
         <v>36000</v>
       </c>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="E15" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="F15" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G15" s="3">
+      <c r="G15" s="2">
         <v>3</v>
       </c>
-      <c r="H15" s="3">
+      <c r="H15" s="2">
         <v>15000</v>
       </c>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="F16" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G16" s="3">
+      <c r="G16" s="2">
         <v>1</v>
       </c>
-      <c r="H16" s="3">
+      <c r="H16" s="2">
         <v>55000</v>
       </c>
     </row>
@@ -2255,373 +2247,331 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P93"/>
+  <dimension ref="A1:I84"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="6" style="2" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="2"/>
+    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="6" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="6" t="s">
         <v>42</v>
       </c>
       <c r="B2" t="s">
         <v>44</v>
       </c>
-      <c r="C2"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3">
         <v>181800</v>
       </c>
-      <c r="C3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4">
         <v>190600</v>
       </c>
-      <c r="C4"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5">
         <v>186200</v>
       </c>
-      <c r="C5"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6">
         <v>558600</v>
       </c>
-      <c r="C6"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7"/>
-      <c r="B7"/>
-      <c r="C7"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="B8" s="16"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="6" t="s">
         <v>42</v>
       </c>
       <c r="B9" t="s">
         <v>44</v>
       </c>
-      <c r="C9"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10">
         <v>27600</v>
       </c>
-      <c r="C10"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="9">
+      <c r="B11">
         <v>456000</v>
       </c>
-      <c r="C11"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="9">
+      <c r="B12">
         <v>75000</v>
       </c>
-      <c r="C12"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B13" s="9">
+      <c r="B13">
         <v>558600</v>
       </c>
-      <c r="C13"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14"/>
-      <c r="B14"/>
-      <c r="C14"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="6" t="s">
         <v>42</v>
       </c>
       <c r="B16" t="s">
         <v>44</v>
       </c>
-      <c r="C16"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
-    </row>
-    <row r="17" spans="1:5">
-      <c r="A17" s="8" t="s">
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="9">
+      <c r="B17">
         <v>60600</v>
       </c>
-      <c r="C17"/>
-    </row>
-    <row r="18" spans="1:5">
-      <c r="A18" s="8" t="s">
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18">
         <v>73800</v>
       </c>
-      <c r="C18"/>
-    </row>
-    <row r="19" spans="1:5">
-      <c r="A19" s="8" t="s">
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B19" s="9">
+      <c r="B19">
         <v>81000</v>
       </c>
-      <c r="C19"/>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="A20" s="8" t="s">
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="9">
+      <c r="B20">
         <v>178200</v>
       </c>
-      <c r="C20"/>
-    </row>
-    <row r="21" spans="1:5">
-      <c r="A21" s="8" t="s">
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="9">
+      <c r="B21">
         <v>165000</v>
       </c>
-      <c r="C21"/>
-    </row>
-    <row r="22" spans="1:5">
-      <c r="A22" s="8" t="s">
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B22" s="9">
+      <c r="B22">
         <v>558600</v>
       </c>
-      <c r="C22"/>
-    </row>
-    <row r="23" spans="1:5">
-      <c r="A23"/>
-      <c r="B23"/>
-      <c r="C23"/>
-    </row>
-    <row r="24" spans="1:5">
-      <c r="A24" s="16" t="s">
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="B24" s="16"/>
-      <c r="C24" s="16"/>
-    </row>
-    <row r="25" spans="1:5">
-      <c r="A25" s="7" t="s">
+      <c r="B24" s="11"/>
+      <c r="C24" s="11"/>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" s="6" t="s">
         <v>42</v>
       </c>
       <c r="B25" t="s">
         <v>48</v>
       </c>
-      <c r="C25"/>
-    </row>
-    <row r="26" spans="1:5">
-      <c r="A26" s="8" t="s">
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B26" s="9">
+      <c r="B26">
         <v>18</v>
       </c>
-      <c r="C26"/>
-    </row>
-    <row r="27" spans="1:5">
-      <c r="A27" s="8" t="s">
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B27" s="9">
+      <c r="B27">
         <v>19</v>
       </c>
-      <c r="C27"/>
-    </row>
-    <row r="28" spans="1:5">
-      <c r="A28" s="8" t="s">
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B28" s="9">
+      <c r="B28">
         <v>14</v>
       </c>
-      <c r="C28"/>
-    </row>
-    <row r="29" spans="1:5">
-      <c r="A29" s="8" t="s">
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B29" s="9">
+      <c r="B29">
         <v>51</v>
       </c>
-      <c r="C29"/>
-    </row>
-    <row r="30" spans="1:5">
-      <c r="A30"/>
-      <c r="B30"/>
-      <c r="C30"/>
-    </row>
-    <row r="31" spans="1:5">
-      <c r="A31" s="16" t="s">
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="B31" s="16"/>
-      <c r="C31" s="16"/>
-    </row>
-    <row r="32" spans="1:5">
-      <c r="A32" s="7" t="s">
+      <c r="B31" s="11"/>
+      <c r="C31" s="11"/>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B32" s="7" t="s">
+      <c r="B32" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="C32"/>
-      <c r="D32"/>
-      <c r="E32"/>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="7" t="s">
+      <c r="A33" s="6" t="s">
         <v>42</v>
       </c>
       <c r="B33" t="s">
@@ -2630,88 +2580,70 @@
       <c r="C33" t="s">
         <v>43</v>
       </c>
-      <c r="D33"/>
-      <c r="E33"/>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="8" t="s">
+      <c r="A34" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B34" s="9">
+      <c r="B34">
         <v>146000</v>
       </c>
-      <c r="C34" s="9">
+      <c r="C34">
         <v>146000</v>
       </c>
-      <c r="D34"/>
-      <c r="E34"/>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="8" t="s">
+      <c r="A35" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B35" s="9">
+      <c r="B35">
         <v>146000</v>
       </c>
-      <c r="C35" s="9">
+      <c r="C35">
         <v>146000</v>
       </c>
-      <c r="D35"/>
-      <c r="E35"/>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="8" t="s">
+      <c r="A36" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B36" s="9">
+      <c r="B36">
         <v>164000</v>
       </c>
-      <c r="C36" s="9">
+      <c r="C36">
         <v>164000</v>
       </c>
-      <c r="D36"/>
-      <c r="E36"/>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="8" t="s">
+      <c r="A37" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B37" s="9">
+      <c r="B37">
         <v>456000</v>
       </c>
-      <c r="C37" s="9">
+      <c r="C37">
         <v>456000</v>
       </c>
-      <c r="D37"/>
-      <c r="E37"/>
-    </row>
-    <row r="38" spans="1:5">
-      <c r="A38"/>
-      <c r="B38"/>
-      <c r="C38"/>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="16" t="s">
+      <c r="A39" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="B39" s="16"/>
-      <c r="C39" s="16"/>
-      <c r="D39" s="16"/>
-      <c r="E39" s="16"/>
+      <c r="B39" s="11"/>
+      <c r="C39" s="11"/>
+      <c r="D39" s="11"/>
+      <c r="E39" s="11"/>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="7" t="s">
+      <c r="A40" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B40" s="7" t="s">
+      <c r="B40" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="C40"/>
-      <c r="D40"/>
-      <c r="E40"/>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="7" t="s">
+      <c r="A41" s="6" t="s">
         <v>42</v>
       </c>
       <c r="B41" t="s">
@@ -2728,118 +2660,111 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="8" t="s">
+      <c r="A42" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B42" s="9">
+      <c r="B42">
         <v>9600</v>
       </c>
-      <c r="C42" s="9">
+      <c r="C42">
         <v>36000</v>
       </c>
-      <c r="D42" s="9">
+      <c r="D42">
         <v>15000</v>
       </c>
-      <c r="E42" s="9">
+      <c r="E42">
         <v>60600</v>
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="8" t="s">
+      <c r="A43" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B43" s="9">
+      <c r="B43">
         <v>4800</v>
       </c>
-      <c r="C43" s="9">
+      <c r="C43">
         <v>54000</v>
       </c>
-      <c r="D43" s="9">
+      <c r="D43">
         <v>15000</v>
       </c>
-      <c r="E43" s="9">
+      <c r="E43">
         <v>73800</v>
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="8" t="s">
+      <c r="A44" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B44" s="9">
+      <c r="B44">
         <v>6000</v>
       </c>
-      <c r="C44" s="9">
+      <c r="C44">
         <v>55000</v>
       </c>
-      <c r="D44" s="9">
+      <c r="D44">
         <v>20000</v>
       </c>
-      <c r="E44" s="9">
+      <c r="E44">
         <v>81000</v>
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="8" t="s">
+      <c r="A45" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B45" s="9">
+      <c r="B45">
         <v>7200</v>
       </c>
-      <c r="C45" s="9">
+      <c r="C45">
         <v>146000</v>
       </c>
-      <c r="D45" s="9">
+      <c r="D45">
         <v>25000</v>
       </c>
-      <c r="E45" s="9">
+      <c r="E45">
         <v>178200</v>
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="8" t="s">
+      <c r="A46" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B46" s="9"/>
-      <c r="C46" s="9">
+      <c r="C46">
         <v>165000</v>
       </c>
-      <c r="D46" s="9"/>
-      <c r="E46" s="9">
+      <c r="E46">
         <v>165000</v>
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="8" t="s">
+      <c r="A47" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B47" s="9">
+      <c r="B47">
         <v>27600</v>
       </c>
-      <c r="C47" s="9">
+      <c r="C47">
         <v>456000</v>
       </c>
-      <c r="D47" s="9">
+      <c r="D47">
         <v>75000</v>
       </c>
-      <c r="E47" s="9">
+      <c r="E47">
         <v>558600</v>
       </c>
     </row>
-    <row r="48" spans="1:5">
-      <c r="A48"/>
-      <c r="B48"/>
-      <c r="C48"/>
-    </row>
     <row r="49" spans="1:4">
-      <c r="A49" s="16" t="s">
+      <c r="A49" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="B49" s="16"/>
-      <c r="C49" s="16"/>
-      <c r="D49" s="16"/>
+      <c r="B49" s="11"/>
+      <c r="C49" s="11"/>
+      <c r="D49" s="11"/>
     </row>
     <row r="50" spans="1:4">
-      <c r="A50" s="7" t="s">
+      <c r="A50" s="6" t="s">
         <v>42</v>
       </c>
       <c r="B50" t="s">
@@ -2850,200 +2775,157 @@
       </c>
     </row>
     <row r="51" spans="1:4">
-      <c r="A51" s="8" t="s">
+      <c r="A51" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B51" s="9">
+      <c r="B51">
         <v>15</v>
       </c>
-      <c r="C51" s="9">
+      <c r="C51">
         <v>75000</v>
       </c>
     </row>
     <row r="52" spans="1:4">
-      <c r="A52" s="8" t="s">
+      <c r="A52" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B52" s="9">
+      <c r="B52">
         <v>6</v>
       </c>
-      <c r="C52" s="9">
+      <c r="C52">
         <v>330000</v>
       </c>
     </row>
     <row r="53" spans="1:4">
-      <c r="A53" s="8" t="s">
+      <c r="A53" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B53" s="9">
+      <c r="B53">
         <v>7</v>
       </c>
-      <c r="C53" s="9">
+      <c r="C53">
         <v>126000</v>
       </c>
     </row>
     <row r="54" spans="1:4">
-      <c r="A54" s="8" t="s">
+      <c r="A54" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B54" s="9">
+      <c r="B54">
         <v>23</v>
       </c>
-      <c r="C54" s="9">
+      <c r="C54">
         <v>27600</v>
       </c>
     </row>
     <row r="55" spans="1:4">
-      <c r="A55" s="8" t="s">
+      <c r="A55" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B55" s="9">
+      <c r="B55">
         <v>51</v>
       </c>
-      <c r="C55" s="9">
+      <c r="C55">
         <v>558600</v>
       </c>
     </row>
-    <row r="56" spans="1:4">
-      <c r="A56"/>
-      <c r="B56"/>
-      <c r="C56"/>
-    </row>
     <row r="57" spans="1:4">
-      <c r="A57" s="16" t="s">
+      <c r="A57" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="B57" s="16"/>
-      <c r="C57" s="16"/>
-      <c r="D57" s="16"/>
+      <c r="B57" s="11"/>
+      <c r="C57" s="11"/>
+      <c r="D57" s="11"/>
     </row>
     <row r="58" spans="1:4">
-      <c r="A58" s="7" t="s">
+      <c r="A58" s="6" t="s">
         <v>42</v>
       </c>
       <c r="B58" t="s">
         <v>54</v>
       </c>
-      <c r="C58"/>
     </row>
     <row r="59" spans="1:4">
-      <c r="A59" s="8" t="s">
+      <c r="A59" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B59" s="9">
+      <c r="B59">
         <v>3</v>
       </c>
-      <c r="C59"/>
     </row>
     <row r="60" spans="1:4">
-      <c r="A60" s="8" t="s">
+      <c r="A60" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B60" s="9">
+      <c r="B60">
         <v>3</v>
       </c>
-      <c r="C60"/>
     </row>
     <row r="61" spans="1:4">
-      <c r="A61" s="8" t="s">
+      <c r="A61" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B61" s="9">
+      <c r="B61">
         <v>3</v>
       </c>
-      <c r="C61"/>
     </row>
     <row r="62" spans="1:4">
-      <c r="A62" s="8" t="s">
+      <c r="A62" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B62" s="9">
+      <c r="B62">
         <v>4</v>
       </c>
-      <c r="C62"/>
     </row>
     <row r="63" spans="1:4">
-      <c r="A63" s="8" t="s">
+      <c r="A63" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B63" s="9">
+      <c r="B63">
         <v>2</v>
       </c>
-      <c r="C63"/>
     </row>
     <row r="64" spans="1:4">
-      <c r="A64" s="8" t="s">
+      <c r="A64" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B64" s="9">
+      <c r="B64">
         <v>15</v>
       </c>
-      <c r="C64"/>
-    </row>
-    <row r="65" spans="1:16">
-      <c r="A65"/>
-      <c r="B65"/>
-      <c r="C65"/>
-    </row>
-    <row r="66" spans="1:16">
-      <c r="A66" s="17" t="s">
+    </row>
+    <row r="66" spans="1:9">
+      <c r="A66" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="B66" s="17"/>
-      <c r="C66" s="17"/>
-      <c r="D66" s="17"/>
-      <c r="E66" s="17"/>
-    </row>
-    <row r="67" spans="1:16">
-      <c r="A67"/>
-      <c r="B67" s="7" t="s">
+      <c r="B66" s="12"/>
+      <c r="C66" s="12"/>
+      <c r="D66" s="12"/>
+      <c r="E66" s="12"/>
+    </row>
+    <row r="67" spans="1:9">
+      <c r="B67" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="C67"/>
-      <c r="D67"/>
-      <c r="E67"/>
-      <c r="F67"/>
-      <c r="G67"/>
-      <c r="H67"/>
-      <c r="I67"/>
-      <c r="J67"/>
-      <c r="K67"/>
-      <c r="L67"/>
-      <c r="M67"/>
-      <c r="N67"/>
-      <c r="O67"/>
-      <c r="P67"/>
-    </row>
-    <row r="68" spans="1:16">
-      <c r="A68"/>
+    </row>
+    <row r="68" spans="1:9">
       <c r="B68" t="s">
         <v>15</v>
       </c>
-      <c r="C68"/>
       <c r="D68" t="s">
         <v>10</v>
       </c>
-      <c r="E68"/>
       <c r="F68" t="s">
         <v>20</v>
       </c>
-      <c r="G68"/>
       <c r="H68" t="s">
         <v>57</v>
       </c>
       <c r="I68" t="s">
         <v>56</v>
       </c>
-      <c r="J68"/>
-      <c r="K68"/>
-      <c r="L68"/>
-      <c r="M68"/>
-      <c r="N68"/>
-      <c r="O68"/>
-      <c r="P68"/>
-    </row>
-    <row r="69" spans="1:16">
-      <c r="A69" s="7" t="s">
+    </row>
+    <row r="69" spans="1:9">
+      <c r="A69" s="6" t="s">
         <v>42</v>
       </c>
       <c r="B69" t="s">
@@ -3064,479 +2946,276 @@
       <c r="G69" t="s">
         <v>44</v>
       </c>
-      <c r="H69"/>
-      <c r="I69"/>
-      <c r="J69"/>
-      <c r="K69"/>
-      <c r="L69"/>
-      <c r="M69"/>
-      <c r="N69"/>
-      <c r="O69"/>
-      <c r="P69"/>
-    </row>
-    <row r="70" spans="1:16">
-      <c r="A70" s="8" t="s">
+    </row>
+    <row r="70" spans="1:9">
+      <c r="A70" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B70" s="9">
+      <c r="B70">
         <v>9</v>
       </c>
-      <c r="C70" s="9">
+      <c r="C70">
         <v>10800</v>
       </c>
-      <c r="D70" s="9">
+      <c r="D70">
         <v>8</v>
       </c>
-      <c r="E70" s="9">
+      <c r="E70">
         <v>9600</v>
       </c>
-      <c r="F70" s="9">
+      <c r="F70">
         <v>6</v>
       </c>
-      <c r="G70" s="9">
+      <c r="G70">
         <v>7200</v>
       </c>
-      <c r="H70" s="9">
+      <c r="H70">
         <v>23</v>
       </c>
-      <c r="I70" s="9">
+      <c r="I70">
         <v>27600</v>
       </c>
-      <c r="J70"/>
-      <c r="K70"/>
-      <c r="L70"/>
-      <c r="M70"/>
-      <c r="N70"/>
-      <c r="O70"/>
-      <c r="P70"/>
-    </row>
-    <row r="71" spans="1:16">
-      <c r="A71" s="8" t="s">
+    </row>
+    <row r="71" spans="1:9">
+      <c r="A71" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B71" s="9">
+      <c r="B71">
         <v>4</v>
       </c>
-      <c r="C71" s="9">
+      <c r="C71">
         <v>146000</v>
       </c>
-      <c r="D71" s="9">
+      <c r="D71">
         <v>4</v>
       </c>
-      <c r="E71" s="9">
+      <c r="E71">
         <v>146000</v>
       </c>
-      <c r="F71" s="9">
+      <c r="F71">
         <v>5</v>
       </c>
-      <c r="G71" s="9">
+      <c r="G71">
         <v>164000</v>
       </c>
-      <c r="H71" s="9">
+      <c r="H71">
         <v>13</v>
       </c>
-      <c r="I71" s="9">
+      <c r="I71">
         <v>456000</v>
       </c>
-      <c r="J71"/>
-      <c r="K71"/>
-      <c r="L71"/>
-      <c r="M71"/>
-      <c r="N71"/>
-      <c r="O71"/>
-      <c r="P71"/>
-    </row>
-    <row r="72" spans="1:16">
-      <c r="A72" s="8" t="s">
+    </row>
+    <row r="72" spans="1:9">
+      <c r="A72" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B72" s="9">
+      <c r="B72">
         <v>5</v>
       </c>
-      <c r="C72" s="9">
+      <c r="C72">
         <v>25000</v>
       </c>
-      <c r="D72" s="9">
+      <c r="D72">
         <v>7</v>
       </c>
-      <c r="E72" s="9">
+      <c r="E72">
         <v>35000</v>
       </c>
-      <c r="F72" s="9">
+      <c r="F72">
         <v>3</v>
       </c>
-      <c r="G72" s="9">
+      <c r="G72">
         <v>15000</v>
       </c>
-      <c r="H72" s="9">
+      <c r="H72">
         <v>15</v>
       </c>
-      <c r="I72" s="9">
+      <c r="I72">
         <v>75000</v>
       </c>
-      <c r="J72"/>
-      <c r="K72"/>
-      <c r="L72"/>
-      <c r="M72"/>
-      <c r="N72"/>
-      <c r="O72"/>
-      <c r="P72"/>
-    </row>
-    <row r="73" spans="1:16">
-      <c r="A73" s="8" t="s">
+    </row>
+    <row r="73" spans="1:9">
+      <c r="A73" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B73" s="9">
+      <c r="B73">
         <v>18</v>
       </c>
-      <c r="C73" s="9">
+      <c r="C73">
         <v>181800</v>
       </c>
-      <c r="D73" s="9">
+      <c r="D73">
         <v>19</v>
       </c>
-      <c r="E73" s="9">
+      <c r="E73">
         <v>190600</v>
       </c>
-      <c r="F73" s="9">
+      <c r="F73">
         <v>14</v>
       </c>
-      <c r="G73" s="9">
+      <c r="G73">
         <v>186200</v>
       </c>
-      <c r="H73" s="9">
+      <c r="H73">
         <v>51</v>
       </c>
-      <c r="I73" s="9">
+      <c r="I73">
         <v>558600</v>
       </c>
-      <c r="J73"/>
-      <c r="K73"/>
-      <c r="L73"/>
-      <c r="M73"/>
-      <c r="N73"/>
-      <c r="O73"/>
-      <c r="P73"/>
-    </row>
-    <row r="74" spans="1:16">
-      <c r="A74"/>
-      <c r="B74"/>
-      <c r="C74"/>
-      <c r="D74"/>
-      <c r="E74"/>
-      <c r="F74"/>
-      <c r="G74"/>
-      <c r="H74"/>
-      <c r="I74"/>
-      <c r="J74"/>
-      <c r="K74"/>
-      <c r="L74"/>
-      <c r="M74"/>
-      <c r="N74"/>
-      <c r="O74"/>
-      <c r="P74"/>
-    </row>
-    <row r="75" spans="1:16">
-      <c r="A75" s="16" t="s">
+    </row>
+    <row r="75" spans="1:9">
+      <c r="A75" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="B75" s="16"/>
-      <c r="C75" s="16"/>
-      <c r="D75" s="16"/>
-      <c r="E75"/>
-      <c r="F75"/>
-      <c r="G75"/>
-      <c r="H75"/>
-      <c r="I75"/>
-      <c r="J75"/>
-      <c r="K75"/>
-      <c r="L75"/>
-      <c r="M75"/>
-      <c r="N75"/>
-      <c r="O75"/>
-      <c r="P75"/>
-    </row>
-    <row r="76" spans="1:16">
-      <c r="A76" s="7" t="s">
+      <c r="B75" s="11"/>
+      <c r="C75" s="11"/>
+      <c r="D75" s="11"/>
+    </row>
+    <row r="76" spans="1:9">
+      <c r="A76" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B76" s="7" t="s">
+      <c r="B76" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="C76"/>
-      <c r="D76"/>
-      <c r="E76"/>
-      <c r="F76"/>
-      <c r="G76"/>
-      <c r="H76"/>
-      <c r="I76"/>
-      <c r="J76"/>
-      <c r="K76"/>
-      <c r="L76"/>
-      <c r="M76"/>
-      <c r="N76"/>
-      <c r="O76"/>
-      <c r="P76"/>
-    </row>
-    <row r="77" spans="1:16">
-      <c r="A77" s="7" t="s">
+    </row>
+    <row r="77" spans="1:9">
+      <c r="A77" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="B77" s="8" t="s">
+      <c r="B77" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C77" s="8" t="s">
+      <c r="C77" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D77" s="8" t="s">
+      <c r="D77" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="E77" s="8" t="s">
+      <c r="E77" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="F77"/>
-      <c r="G77"/>
-      <c r="H77"/>
-      <c r="I77"/>
-      <c r="J77"/>
-      <c r="K77"/>
-      <c r="L77"/>
-      <c r="M77"/>
-      <c r="N77"/>
-      <c r="O77"/>
-      <c r="P77"/>
-    </row>
-    <row r="78" spans="1:16">
-      <c r="A78" s="8" t="s">
+    </row>
+    <row r="78" spans="1:9">
+      <c r="A78" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B78" s="11">
+      <c r="B78" s="7">
         <v>36000</v>
       </c>
-      <c r="C78" s="11">
+      <c r="C78" s="7">
         <v>9600</v>
       </c>
-      <c r="D78" s="11">
+      <c r="D78" s="7">
         <v>15000</v>
       </c>
-      <c r="E78" s="11">
+      <c r="E78" s="7">
         <v>60600</v>
       </c>
-      <c r="F78"/>
-      <c r="G78"/>
-      <c r="H78"/>
-      <c r="I78"/>
-      <c r="J78"/>
-      <c r="K78"/>
-      <c r="L78"/>
-      <c r="M78"/>
-      <c r="N78"/>
-      <c r="O78"/>
-      <c r="P78"/>
-    </row>
-    <row r="79" spans="1:16">
-      <c r="A79" s="8" t="s">
+    </row>
+    <row r="79" spans="1:9">
+      <c r="A79" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B79" s="11">
+      <c r="B79" s="7">
         <v>4800</v>
       </c>
-      <c r="C79" s="11">
+      <c r="C79" s="7">
         <v>15000</v>
       </c>
-      <c r="D79" s="11">
+      <c r="D79" s="7">
         <v>54000</v>
       </c>
-      <c r="E79" s="11">
+      <c r="E79" s="7">
         <v>73800</v>
       </c>
-      <c r="F79"/>
-      <c r="G79"/>
-      <c r="H79"/>
-      <c r="I79"/>
-      <c r="J79"/>
-      <c r="K79"/>
-      <c r="L79"/>
-      <c r="M79"/>
-      <c r="N79"/>
-      <c r="O79"/>
-      <c r="P79"/>
-    </row>
-    <row r="80" spans="1:16">
-      <c r="A80" s="8" t="s">
+    </row>
+    <row r="80" spans="1:9">
+      <c r="A80" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B80" s="11">
+      <c r="B80" s="7">
         <v>6000</v>
       </c>
-      <c r="C80" s="11">
+      <c r="C80" s="7">
         <v>20000</v>
       </c>
-      <c r="D80" s="11">
+      <c r="D80" s="7">
         <v>55000</v>
       </c>
-      <c r="E80" s="11">
+      <c r="E80" s="7">
         <v>81000</v>
       </c>
-      <c r="F80"/>
-      <c r="G80"/>
-      <c r="H80"/>
-      <c r="I80"/>
-      <c r="J80"/>
-      <c r="K80"/>
-      <c r="L80"/>
-      <c r="M80"/>
-      <c r="N80"/>
-      <c r="O80"/>
-      <c r="P80"/>
-    </row>
-    <row r="81" spans="1:16">
-      <c r="A81" s="8" t="s">
+    </row>
+    <row r="81" spans="1:5">
+      <c r="A81" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B81" s="11">
+      <c r="B81" s="7">
         <v>25000</v>
       </c>
-      <c r="C81" s="11">
+      <c r="C81" s="7">
         <v>146000</v>
       </c>
-      <c r="D81" s="11">
+      <c r="D81" s="7">
         <v>7200</v>
       </c>
-      <c r="E81" s="11">
+      <c r="E81" s="7">
         <v>178200</v>
       </c>
-      <c r="F81"/>
-      <c r="G81"/>
-      <c r="H81"/>
-      <c r="I81"/>
-      <c r="J81"/>
-      <c r="K81"/>
-      <c r="L81"/>
-      <c r="M81"/>
-      <c r="N81"/>
-      <c r="O81"/>
-      <c r="P81"/>
-    </row>
-    <row r="82" spans="1:16">
-      <c r="A82" s="8" t="s">
+    </row>
+    <row r="82" spans="1:5">
+      <c r="A82" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B82" s="11">
+      <c r="B82" s="7">
         <v>110000</v>
       </c>
-      <c r="C82" s="11"/>
-      <c r="D82" s="11">
+      <c r="C82" s="7"/>
+      <c r="D82" s="7">
         <v>55000</v>
       </c>
-      <c r="E82" s="11">
+      <c r="E82" s="7">
         <v>165000</v>
       </c>
-      <c r="F82"/>
-      <c r="G82"/>
-      <c r="H82"/>
-      <c r="I82"/>
-      <c r="J82"/>
-      <c r="K82"/>
-      <c r="L82"/>
-      <c r="M82"/>
-      <c r="N82"/>
-      <c r="O82"/>
-      <c r="P82"/>
-    </row>
-    <row r="83" spans="1:16">
-      <c r="A83" s="8" t="s">
+    </row>
+    <row r="83" spans="1:5">
+      <c r="A83" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B83" s="9">
+      <c r="B83">
         <v>181800</v>
       </c>
-      <c r="C83" s="9">
+      <c r="C83">
         <v>190600</v>
       </c>
-      <c r="D83" s="9">
+      <c r="D83">
         <v>186200</v>
       </c>
-      <c r="E83" s="9">
+      <c r="E83">
         <v>558600</v>
       </c>
-      <c r="F83"/>
-      <c r="G83"/>
-      <c r="H83"/>
-      <c r="I83"/>
-      <c r="J83"/>
-      <c r="K83"/>
-      <c r="L83"/>
-      <c r="M83"/>
-      <c r="N83"/>
-      <c r="O83"/>
-      <c r="P83"/>
-    </row>
-    <row r="84" spans="1:16">
-      <c r="A84" s="10" t="s">
+    </row>
+    <row r="84" spans="1:5">
+      <c r="A84" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="B84" s="10"/>
-      <c r="C84" s="10"/>
-    </row>
-    <row r="85" spans="1:16">
-      <c r="A85"/>
-      <c r="B85"/>
-      <c r="C85"/>
-    </row>
-    <row r="86" spans="1:16">
-      <c r="A86"/>
-      <c r="B86"/>
-      <c r="C86"/>
-    </row>
-    <row r="87" spans="1:16">
-      <c r="A87"/>
-      <c r="B87"/>
-      <c r="C87"/>
-    </row>
-    <row r="88" spans="1:16">
-      <c r="A88"/>
-      <c r="B88"/>
-      <c r="C88"/>
-    </row>
-    <row r="89" spans="1:16">
-      <c r="A89"/>
-      <c r="B89"/>
-      <c r="C89"/>
-    </row>
-    <row r="90" spans="1:16">
-      <c r="A90"/>
-      <c r="B90"/>
-      <c r="C90"/>
-    </row>
-    <row r="91" spans="1:16">
-      <c r="A91"/>
-      <c r="B91"/>
-      <c r="C91"/>
-    </row>
-    <row r="92" spans="1:16">
-      <c r="A92"/>
-      <c r="B92"/>
-      <c r="C92"/>
-    </row>
-    <row r="93" spans="1:16">
-      <c r="A93"/>
-      <c r="B93"/>
-      <c r="C93"/>
+      <c r="B84" s="13"/>
+      <c r="C84" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A31:C31"/>
     <mergeCell ref="A49:D49"/>
     <mergeCell ref="A57:D57"/>
     <mergeCell ref="A66:E66"/>
     <mergeCell ref="A75:D75"/>
     <mergeCell ref="A84:C84"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="A39:E39"/>
   </mergeCells>
   <conditionalFormatting pivot="1" sqref="C51:C54">
     <cfRule type="dataBar" priority="2">
@@ -3607,17 +3286,17 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:1" ht="31.5">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="8" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="18">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="4" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:1">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -3627,17 +3306,17 @@
       </c>
     </row>
     <row r="8" spans="1:1" ht="18">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="4" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="10" spans="1:1">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="5" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="12" spans="1:1" ht="18">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="4" t="s">
         <v>66</v>
       </c>
     </row>
@@ -3672,17 +3351,17 @@
       </c>
     </row>
     <row r="26" spans="1:1" ht="18">
-      <c r="A26" s="5" t="s">
+      <c r="A26" s="4" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="28" spans="1:1">
-      <c r="A28" s="6" t="s">
+      <c r="A28" s="5" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="29" spans="1:1">
-      <c r="A29" s="6" t="s">
+      <c r="A29" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -3692,89 +3371,89 @@
       </c>
     </row>
     <row r="32" spans="1:1">
-      <c r="A32" s="13"/>
+      <c r="A32" s="9"/>
     </row>
     <row r="33" spans="1:1">
-      <c r="A33" s="14" t="s">
+      <c r="A33" s="10" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="34" spans="1:1">
-      <c r="A34" s="14" t="s">
+      <c r="A34" s="10" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="35" spans="1:1">
-      <c r="A35" s="13"/>
+      <c r="A35" s="9"/>
     </row>
     <row r="36" spans="1:1">
-      <c r="A36" s="13" t="s">
+      <c r="A36" s="9" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="38" spans="1:1" ht="18">
-      <c r="A38" s="5" t="s">
+      <c r="A38" s="4" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="39" spans="1:1">
-      <c r="A39" s="13"/>
+      <c r="A39" s="9"/>
     </row>
     <row r="40" spans="1:1">
-      <c r="A40" s="13" t="s">
+      <c r="A40" s="9" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="41" spans="1:1">
-      <c r="A41" s="13" t="s">
+      <c r="A41" s="9" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="42" spans="1:1">
-      <c r="A42" s="13" t="s">
+      <c r="A42" s="9" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="43" spans="1:1">
-      <c r="A43" s="13" t="s">
+      <c r="A43" s="9" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="44" spans="1:1">
-      <c r="A44" s="13" t="s">
+      <c r="A44" s="9" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="45" spans="1:1">
-      <c r="A45" s="13" t="s">
+      <c r="A45" s="9" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="46" spans="1:1">
-      <c r="A46" s="13" t="s">
+      <c r="A46" s="9" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="47" spans="1:1">
-      <c r="A47" s="13" t="s">
+      <c r="A47" s="9" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="48" spans="1:1">
-      <c r="A48" s="13" t="s">
+      <c r="A48" s="9" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="50" spans="1:1" ht="18">
-      <c r="A50" s="5" t="s">
+      <c r="A50" s="4" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="51" spans="1:1">
-      <c r="A51" s="13"/>
+      <c r="A51" s="9"/>
     </row>
     <row r="52" spans="1:1">
-      <c r="A52" s="14" t="s">
+      <c r="A52" s="10" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>